<commit_message>
adding new istallation and run files to git
</commit_message>
<xml_diff>
--- a/data/main.xlsx
+++ b/data/main.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="AppInfo" sheetId="1" state="visible" r:id="rId3"/>
@@ -49,7 +49,9 @@
     <t xml:space="preserve">changelog</t>
   </si>
   <si>
-    <t xml:space="preserve">- Initial Arch Linux setup\n- Added Firebase sync\n- Fixed .desktop launcher</t>
+    <t xml:space="preserve">- Initial Arch Linux setup
+- Added Firebase sync
+- Fixed .desktop launcher</t>
   </si>
   <si>
     <t xml:space="preserve">developer</t>
@@ -5283,7 +5285,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5293,7 +5295,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD4EA6B"/>
-        <bgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFBBE33D"/>
       </patternFill>
     </fill>
     <fill>
@@ -5336,6 +5338,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFD7"/>
         <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBBE33D"/>
+        <bgColor rgb="FFD4EA6B"/>
       </patternFill>
     </fill>
   </fills>
@@ -5386,7 +5394,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="137">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5891,8 +5899,48 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="10" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -5906,7 +5954,7 @@
     <cellStyle name="Untitled1" xfId="21"/>
     <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -6020,6 +6068,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFBBE33D"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFD9EAD3"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -6094,7 +6150,7 @@
       <rgbColor rgb="FFFCE5CD"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFBBE33D"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -6328,7 +6384,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -37092,7 +37148,7 @@
       <c r="E42" s="70" t="s">
         <v>431</v>
       </c>
-      <c r="F42" s="71" t="s">
+      <c r="F42" s="70" t="s">
         <v>432</v>
       </c>
       <c r="G42" s="68"/>
@@ -43117,174 +43173,174 @@
       <c r="I336" s="112"/>
       <c r="J336" s="112"/>
     </row>
-    <row r="337" customFormat="false" ht="165" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A337" s="68" t="s">
+    <row r="337" s="128" customFormat="true" ht="165" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A337" s="126" t="s">
         <v>306</v>
       </c>
-      <c r="B337" s="69" t="n">
+      <c r="B337" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="C337" s="53" t="s">
+      <c r="C337" s="128" t="s">
         <v>1036</v>
       </c>
-      <c r="E337" s="54" t="s">
+      <c r="E337" s="129" t="s">
         <v>1037</v>
       </c>
-      <c r="I337" s="103" t="s">
+      <c r="I337" s="130" t="s">
         <v>1038</v>
       </c>
     </row>
-    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A338" s="68" t="s">
+    <row r="338" s="128" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A338" s="126" t="s">
         <v>306</v>
       </c>
-      <c r="B338" s="69" t="n">
+      <c r="B338" s="127" t="n">
         <v>2</v>
       </c>
-      <c r="C338" s="53" t="s">
+      <c r="C338" s="128" t="s">
         <v>1039</v>
       </c>
-      <c r="D338" s="53" t="s">
+      <c r="D338" s="128" t="s">
         <v>1040</v>
       </c>
-      <c r="E338" s="54" t="s">
+      <c r="E338" s="129" t="s">
         <v>1041</v>
       </c>
-      <c r="H338" s="104" t="s">
+      <c r="H338" s="131" t="s">
         <v>1042</v>
       </c>
-      <c r="I338" s="53" t="s">
+      <c r="I338" s="128" t="s">
         <v>1043</v>
       </c>
     </row>
-    <row r="339" customFormat="false" ht="132.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A339" s="68" t="s">
+    <row r="339" s="128" customFormat="true" ht="132.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A339" s="126" t="s">
         <v>306</v>
       </c>
-      <c r="B339" s="69" t="n">
+      <c r="B339" s="127" t="n">
         <v>3</v>
       </c>
-      <c r="D339" s="53" t="s">
+      <c r="D339" s="128" t="s">
         <v>1044</v>
       </c>
-      <c r="E339" s="54" t="s">
+      <c r="E339" s="129" t="s">
         <v>1045</v>
       </c>
-      <c r="F339" s="103" t="s">
+      <c r="F339" s="130" t="s">
         <v>1046</v>
       </c>
     </row>
-    <row r="340" customFormat="false" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A340" s="68" t="s">
+    <row r="340" s="128" customFormat="true" ht="34.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A340" s="126" t="s">
         <v>311</v>
       </c>
-      <c r="B340" s="69" t="n">
+      <c r="B340" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="C340" s="68" t="s">
+      <c r="C340" s="126" t="s">
         <v>1047</v>
       </c>
-      <c r="D340" s="68" t="s">
+      <c r="D340" s="126" t="s">
         <v>1048</v>
       </c>
-      <c r="E340" s="70" t="s">
+      <c r="E340" s="132" t="s">
         <v>1049</v>
       </c>
-      <c r="F340" s="71" t="s">
+      <c r="F340" s="133" t="s">
         <v>1050</v>
       </c>
-      <c r="G340" s="68"/>
-      <c r="H340" s="68" t="s">
+      <c r="G340" s="126"/>
+      <c r="H340" s="126" t="s">
         <v>1051</v>
       </c>
-      <c r="I340" s="68"/>
-      <c r="J340" s="68"/>
-    </row>
-    <row r="341" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A341" s="68" t="s">
+      <c r="I340" s="126"/>
+      <c r="J340" s="126"/>
+    </row>
+    <row r="341" s="128" customFormat="true" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A341" s="126" t="s">
         <v>311</v>
       </c>
-      <c r="B341" s="69" t="n">
+      <c r="B341" s="127" t="n">
         <v>2</v>
       </c>
-      <c r="C341" s="68"/>
-      <c r="D341" s="68"/>
-      <c r="E341" s="70" t="s">
+      <c r="C341" s="126"/>
+      <c r="D341" s="126"/>
+      <c r="E341" s="132" t="s">
         <v>1052</v>
       </c>
-      <c r="F341" s="71" t="s">
+      <c r="F341" s="133" t="s">
         <v>1053</v>
       </c>
-      <c r="G341" s="68"/>
-      <c r="H341" s="68"/>
-      <c r="I341" s="68"/>
-      <c r="J341" s="68"/>
-    </row>
-    <row r="342" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A342" s="68" t="s">
+      <c r="G341" s="126"/>
+      <c r="H341" s="126"/>
+      <c r="I341" s="126"/>
+      <c r="J341" s="126"/>
+    </row>
+    <row r="342" s="134" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A342" s="126" t="s">
         <v>311</v>
       </c>
-      <c r="B342" s="69" t="n">
+      <c r="B342" s="127" t="n">
         <v>3</v>
       </c>
-      <c r="C342" s="68"/>
-      <c r="D342" s="68"/>
-      <c r="E342" s="70" t="s">
+      <c r="C342" s="126"/>
+      <c r="D342" s="126"/>
+      <c r="E342" s="132" t="s">
         <v>1054</v>
       </c>
-      <c r="F342" s="71" t="s">
+      <c r="F342" s="133" t="s">
         <v>1055</v>
       </c>
-      <c r="G342" s="68"/>
-      <c r="H342" s="68" t="s">
+      <c r="G342" s="126"/>
+      <c r="H342" s="126" t="s">
         <v>1056</v>
       </c>
-      <c r="I342" s="68"/>
-      <c r="J342" s="68"/>
-    </row>
-    <row r="343" s="1" customFormat="true" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A343" s="68" t="s">
+      <c r="I342" s="126"/>
+      <c r="J342" s="126"/>
+    </row>
+    <row r="343" s="134" customFormat="true" ht="45.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A343" s="126" t="s">
         <v>311</v>
       </c>
-      <c r="B343" s="69" t="n">
+      <c r="B343" s="127" t="n">
         <v>4</v>
       </c>
-      <c r="C343" s="68"/>
-      <c r="D343" s="68" t="s">
+      <c r="C343" s="126"/>
+      <c r="D343" s="126" t="s">
         <v>1057</v>
       </c>
-      <c r="E343" s="70" t="s">
+      <c r="E343" s="132" t="s">
         <v>1058</v>
       </c>
-      <c r="F343" s="71"/>
-      <c r="G343" s="68"/>
-      <c r="H343" s="68"/>
-      <c r="I343" s="68"/>
-      <c r="J343" s="68"/>
-    </row>
-    <row r="344" s="1" customFormat="true" ht="77.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A344" s="68" t="s">
+      <c r="F343" s="133"/>
+      <c r="G343" s="126"/>
+      <c r="H343" s="126"/>
+      <c r="I343" s="126"/>
+      <c r="J343" s="126"/>
+    </row>
+    <row r="344" s="134" customFormat="true" ht="77.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A344" s="126" t="s">
         <v>311</v>
       </c>
-      <c r="B344" s="69" t="n">
+      <c r="B344" s="127" t="n">
         <v>5</v>
       </c>
-      <c r="C344" s="68"/>
-      <c r="D344" s="68" t="s">
+      <c r="C344" s="126"/>
+      <c r="D344" s="126" t="s">
         <v>1059</v>
       </c>
-      <c r="E344" s="70" t="s">
+      <c r="E344" s="132" t="s">
         <v>1060</v>
       </c>
-      <c r="F344" s="126" t="s">
+      <c r="F344" s="135" t="s">
         <v>1061</v>
       </c>
-      <c r="G344" s="68"/>
-      <c r="H344" s="68"/>
-      <c r="I344" s="73" t="s">
+      <c r="G344" s="126"/>
+      <c r="H344" s="126"/>
+      <c r="I344" s="136" t="s">
         <v>1062</v>
       </c>
-      <c r="J344" s="68"/>
+      <c r="J344" s="126"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J344">

</xml_diff>